<commit_message>
Rename proposal change log to BC Bid Log and add estimator link
Rename "Change Log" to "BC Bid Log" in ProjectLogPage, AdminPage, and update tab labels. Add "Estimator" link to Header.tsx toolRoutes and conditionally hide the "Estimate" button on the "BC Bid Log" tab.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 58930b83-e729-431e-b4fb-7d5f1e2c27e8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/sD6xXyi
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="108">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>HK</t>
   </si>
   <si>
     <t>Nilda Puno</t>
@@ -1294,10 +1297,10 @@
         <v>93</v>
       </c>
       <c r="G13" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="H13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" t="s">
         <v>17</v>
@@ -1315,33 +1318,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1359,18 +1362,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" t="s">
         <v>76</v>
@@ -1385,7 +1388,7 @@
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I15" t="s">
         <v>17</v>
@@ -1403,7 +1406,7 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a way to view estimate details from the proposal log
Add a new button to the proposal log that links to the estimate details.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a7d3985c-bf9e-48f5-9f96-3555cbeae2f1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/sD6xXyi
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -274,6 +274,9 @@
     <t>2026-04-21</t>
   </si>
   <si>
+    <t>HK</t>
+  </si>
+  <si>
     <t>Vahid Balali</t>
   </si>
   <si>
@@ -293,9 +296,6 @@
   </si>
   <si>
     <t>2026-04-11</t>
-  </si>
-  <si>
-    <t>HK</t>
   </si>
   <si>
     <t>Nilda Puno</t>
@@ -1253,10 +1253,10 @@
         <v>86</v>
       </c>
       <c r="G12" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="H12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I12" t="s">
         <v>17</v>
@@ -1274,30 +1274,30 @@
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G13" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>95</v>

</xml_diff>

<commit_message>
Enhance proposal log with new filtering and role-based views
Update ProjectLogPage.tsx to include role-based filtering (Leadership/Estimator), region and status filters, and adjust the visibility of the "Estimate" button based on proposal status.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1389662b-2bad-48dd-8dbb-b7d5cb282bc8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/mmTy3QM
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="109">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -332,6 +332,9 @@
   </si>
   <si>
     <t>DeShaun Taylor</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
@@ -1391,7 +1394,7 @@
         <v>106</v>
       </c>
       <c r="I15" t="s">
-        <v>17</v>
+        <v>107</v>
       </c>
       <c r="J15" t="s">
         <v>56</v>
@@ -1406,7 +1409,7 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add estimate links to project bids and include "Lead" status
Update the home page HUD to include a calculator icon link for bids with "Lead" or "Estimating" statuses, allowing direct access to the estimating module.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 97d19c88-24fc-4107-a6c5-79bdb4b8e774
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/mmTy3QM
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="111">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -338,6 +338,12 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
+  </si>
+  <si>
+    <t>26-0217</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
   </si>
 </sst>
 </file>
@@ -736,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1412,8 +1418,52 @@
         <v>108</v>
       </c>
     </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" t="s">
+        <v>86</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>106</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>56</v>
+      </c>
+      <c r="K16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:N16"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update project details and scope selection for better proposal management
Implement bi-directional syncing for project information and scope selections between the proposal log and estimate modules, and refine the scope list in the estimate module to exclude specific items.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 35146166-2a8d-43fd-84ae-34c1f72199a6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/H1Y8NMj
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -280,6 +280,9 @@
     <t>Vahid Balali</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
   </si>
   <si>
@@ -332,9 +335,6 @@
   </si>
   <si>
     <t>DeShaun Taylor</t>
-  </si>
-  <si>
-    <t>0</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
@@ -1268,7 +1268,7 @@
         <v>88</v>
       </c>
       <c r="I12" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="J12" t="s">
         <v>56</v>
@@ -1283,36 +1283,36 @@
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="H13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I13" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="J13" t="s">
         <v>56</v>
@@ -1327,33 +1327,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1371,18 +1371,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
         <v>76</v>
@@ -1397,10 +1397,10 @@
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I15" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="J15" t="s">
         <v>56</v>
@@ -1423,10 +1423,10 @@
         <v>109</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" t="s">
         <v>76</v>
@@ -1441,7 +1441,7 @@
         <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I16" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Improve data synchronization and field consistency between proposal and estimate modules
Synchronizes Region and Status dropdowns, fixes scope sync for existing estimates, and updates date field formatting in the Estimating Module.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 79ab2b16-032c-4589-b119-106c51551be6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/Yw5EduY
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="113">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -281,6 +281,12 @@
   </si>
   <si>
     <t>0</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>2026-11-01</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
@@ -1274,42 +1280,42 @@
         <v>56</v>
       </c>
       <c r="K12" t="s">
-        <v>17</v>
+        <v>90</v>
       </c>
       <c r="L12" t="s">
-        <v>17</v>
+        <v>91</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G13" t="s">
         <v>82</v>
       </c>
       <c r="H13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I13" t="s">
         <v>89</v>
@@ -1327,33 +1333,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1371,18 +1377,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
         <v>76</v>
@@ -1397,7 +1403,7 @@
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I15" t="s">
         <v>89</v>
@@ -1415,18 +1421,18 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D16" t="s">
         <v>76</v>
@@ -1441,7 +1447,7 @@
         <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I16" t="s">
         <v>17</v>
@@ -1459,7 +1465,7 @@
         <v>17</v>
       </c>
       <c r="N16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update proposal log backup file with current data
Backup file for the proposal log has been updated with recent entries.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a4ca6b83-df37-4850-a7ea-6ca5745c7339
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/jotkESu
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -181,6 +181,9 @@
     <t>Nick Jennings</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Estimating</t>
   </si>
   <si>
@@ -278,9 +281,6 @@
   </si>
   <si>
     <t>Vahid Balali</t>
-  </si>
-  <si>
-    <t>0</t>
   </si>
   <si>
     <t>2026-06-01</t>
@@ -1010,10 +1010,10 @@
         <v>55</v>
       </c>
       <c r="I6" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="J6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K6" t="s">
         <v>17</v>
@@ -1025,18 +1025,18 @@
         <v>17</v>
       </c>
       <c r="N6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
         <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
         <v>45</v>
@@ -1051,13 +1051,13 @@
         <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I7" t="s">
         <v>17</v>
       </c>
       <c r="J7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K7" t="s">
         <v>17</v>
@@ -1069,18 +1069,18 @@
         <v>17</v>
       </c>
       <c r="N7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -1089,19 +1089,19 @@
         <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
       </c>
       <c r="H8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
         <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K8" t="s">
         <v>17</v>
@@ -1113,15 +1113,15 @@
         <v>17</v>
       </c>
       <c r="N8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
@@ -1133,19 +1133,19 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G9" t="s">
         <v>17</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I9" t="s">
         <v>17</v>
       </c>
       <c r="J9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K9" t="s">
         <v>17</v>
@@ -1157,39 +1157,39 @@
         <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G10" t="s">
         <v>17</v>
       </c>
       <c r="H10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
         <v>17</v>
       </c>
       <c r="J10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K10" t="s">
         <v>17</v>
@@ -1201,12 +1201,12 @@
         <v>17</v>
       </c>
       <c r="N10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
@@ -1224,7 +1224,7 @@
         <v>19</v>
       </c>
       <c r="G11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
@@ -1233,7 +1233,7 @@
         <v>17</v>
       </c>
       <c r="J11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K11" t="s">
         <v>17</v>
@@ -1250,34 +1250,34 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I12" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="J12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K12" t="s">
         <v>90</v>
@@ -1312,16 +1312,16 @@
         <v>97</v>
       </c>
       <c r="G13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H13" t="s">
         <v>98</v>
       </c>
       <c r="I13" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="J13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
@@ -1365,7 +1365,7 @@
         <v>17</v>
       </c>
       <c r="J14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K14" t="s">
         <v>17</v>
@@ -1391,13 +1391,13 @@
         <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
@@ -1406,10 +1406,10 @@
         <v>109</v>
       </c>
       <c r="I15" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="J15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K15" t="s">
         <v>17</v>
@@ -1435,13 +1435,13 @@
         <v>108</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
         <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G16" t="s">
         <v>17</v>
@@ -1453,7 +1453,7 @@
         <v>17</v>
       </c>
       <c r="J16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K16" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Improve print functionality for proposals to create cleaner documents
Update the print button to invoke a new `handlePrint` function that generates a clean HTML document for printing proposal details, including custom styles and auto-triggering the browser's print dialog.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: afe673ac-0768-4d76-aafa-b219a00e57de
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/2cZ4QSZ
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-07.xlsx
+++ b/backups/proposal-log-2026-04-07.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="114">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -263,6 +263,9 @@
   </si>
   <si>
     <t>GT</t>
+  </si>
+  <si>
+    <t>10187</t>
   </si>
   <si>
     <t>26-0207</t>
@@ -1230,7 +1233,7 @@
         <v>20</v>
       </c>
       <c r="I11" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="J11" t="s">
         <v>57</v>
@@ -1250,13 +1253,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D12" t="s">
         <v>77</v>
@@ -1265,13 +1268,13 @@
         <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I12" t="s">
         <v>56</v>
@@ -1280,42 +1283,42 @@
         <v>57</v>
       </c>
       <c r="K12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G13" t="s">
         <v>83</v>
       </c>
       <c r="H13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I13" t="s">
         <v>56</v>
@@ -1333,33 +1336,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1377,18 +1380,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
         <v>77</v>
@@ -1397,13 +1400,13 @@
         <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I15" t="s">
         <v>56</v>
@@ -1421,18 +1424,18 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D16" t="s">
         <v>77</v>
@@ -1441,13 +1444,13 @@
         <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G16" t="s">
         <v>17</v>
       </c>
       <c r="H16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I16" t="s">
         <v>17</v>
@@ -1465,7 +1468,7 @@
         <v>17</v>
       </c>
       <c r="N16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>